<commit_message>
Dodano modele STEP214 dennicy górnej i dolnej w wymiarach nominalnych, z wygaszonymi otworami obwodowymi do połączenia z rurą zbiornika.
</commit_message>
<xml_diff>
--- a/Zbiornik/Obliczenia.xlsx
+++ b/Zbiornik/Obliczenia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1wB3C7psRW9DwIbbp428GwwekvqOcbzY-\SimBa\Projekty (dawniej rakiety)\R7\03_Propulsion\Model 3D w SolidWorks\Zbiornik\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SimLE_Git\Main-Assembly\R7_ENG_0000\Zbiornik\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6150BB8C-1FF6-48A8-A16B-64EEB2D52BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF023CBC-5F6A-47DE-8B88-2E04B32E5E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2388" yWindow="324" windowWidth="18420" windowHeight="12816" xr2:uid="{884CEEDE-8FB0-4B0A-BCDA-4E8CBB830B75}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{884CEEDE-8FB0-4B0A-BCDA-4E8CBB830B75}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -685,25 +685,25 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1856,17 +1856,17 @@
       <c r="B1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="14" t="s">
+      <c r="F1" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
+      <c r="N1" s="15"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="F2" t="s">
@@ -1910,14 +1910,14 @@
       </c>
       <c r="B3">
         <f>D3*0.001</f>
-        <v>0.16300000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
       </c>
       <c r="D3">
-        <f>180-2*8.5</f>
-        <v>163</v>
+        <f>180-2*10</f>
+        <v>160</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -1970,14 +1970,14 @@
       </c>
       <c r="B4">
         <f>D4*0.001</f>
-        <v>8.1500000000000003E-2</v>
+        <v>0.08</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
       </c>
       <c r="D4">
         <f>D3/2</f>
-        <v>81.5</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="G10" s="4">
         <f>1000*($B$12*$B$11*$B$4)/(G3-0.6*$B$11)</f>
-        <v>4.7847358121330732</v>
+        <v>4.6966731898238745</v>
       </c>
       <c r="H10" s="1"/>
       <c r="I10" s="1"/>
@@ -2317,31 +2317,31 @@
       </c>
       <c r="G11" s="5">
         <f t="shared" ref="G11:M11" si="6">$D$4+G9</f>
-        <v>86.607632093933461</v>
+        <v>85.107632093933461</v>
       </c>
       <c r="H11" s="5">
         <f t="shared" si="6"/>
-        <v>91.130996309963095</v>
+        <v>89.630996309963095</v>
       </c>
       <c r="I11" s="5">
         <f t="shared" si="6"/>
-        <v>86.92619542619542</v>
+        <v>85.42619542619542</v>
       </c>
       <c r="J11" s="5">
         <f t="shared" si="6"/>
-        <v>87.041401273885356</v>
+        <v>85.541401273885356</v>
       </c>
       <c r="K11" s="5">
         <f t="shared" si="6"/>
-        <v>83.086626139817625</v>
+        <v>81.586626139817625</v>
       </c>
       <c r="L11" s="5">
         <f t="shared" si="6"/>
-        <v>87.699524940617579</v>
+        <v>86.199524940617579</v>
       </c>
       <c r="M11" s="5">
         <f t="shared" si="6"/>
-        <v>86.070928196147108</v>
+        <v>84.570928196147108</v>
       </c>
       <c r="N11" t="s">
         <v>10</v>
@@ -2366,31 +2366,31 @@
       </c>
       <c r="G12" s="4">
         <f>1000*$B$10/(PI()*$B$4^2)</f>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="H12" s="5">
         <f>1000*$B$10/(PI()*$B$4^2)</f>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="I12" s="5">
         <f>1000*$B$10/(PI()*$B$4^2)</f>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="J12" s="5">
         <f>1000*$B$10/(PI()*$B$4^2)</f>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="K12" s="5">
         <f>1000*$B$10/(PI()*$B$4^2)</f>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="L12" s="5">
         <f t="shared" ref="L12:M12" si="7">1000*$B$10/(PI()*$B$4^2)</f>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="M12" s="5">
         <f t="shared" si="7"/>
-        <v>707.57311364719544</v>
+        <v>734.3558615817318</v>
       </c>
       <c r="N12" t="s">
         <v>10</v>
@@ -2431,31 +2431,31 @@
       </c>
       <c r="G13" s="4">
         <f t="shared" ref="G13:M13" si="8">((PI()*G11^2*G12/1000)-(PI()*$D$4^2*G12/1000))*G5*0.000001</f>
-        <v>5.153377977002223</v>
+        <v>5.2529946532925855</v>
       </c>
       <c r="H13" s="5">
         <f t="shared" si="8"/>
-        <v>9.9787226637414346</v>
+        <v>10.176457704623223</v>
       </c>
       <c r="I13" s="5">
         <f t="shared" si="8"/>
-        <v>5.6883236125892376</v>
+        <v>5.7984802520619816</v>
       </c>
       <c r="J13" s="5">
         <f t="shared" si="8"/>
-        <v>5.6054587330654533</v>
+        <v>5.7140814927488064</v>
       </c>
       <c r="K13" s="5">
         <f t="shared" si="8"/>
-        <v>2.5715446470826366</v>
+        <v>2.6202346343378857</v>
       </c>
       <c r="L13" s="5">
         <f t="shared" si="8"/>
-        <v>18.653860849242335</v>
+        <v>19.016676342063178</v>
       </c>
       <c r="M13" s="5">
         <f t="shared" si="8"/>
-        <v>13.621165078457329</v>
+        <v>13.883659153584857</v>
       </c>
       <c r="N13" t="s">
         <v>0</v>
@@ -2507,11 +2507,11 @@
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="F15" s="14" t="s">
+      <c r="F15" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
       <c r="R15">
         <v>14</v>
       </c>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="G16">
         <f>PI()*B4^2</f>
-        <v>2.0867243803306804E-2</v>
+        <v>2.0106192982974676E-2</v>
       </c>
       <c r="H16" t="s">
         <v>38</v>
@@ -2555,7 +2555,7 @@
       </c>
       <c r="G17">
         <f>B11*10^6*G16</f>
-        <v>156504.32852480104</v>
+        <v>150796.44737231007</v>
       </c>
       <c r="H17" t="s">
         <v>40</v>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G18">
         <f>G17/B33</f>
-        <v>37.146891871783012</v>
+        <v>35.792104780670897</v>
       </c>
       <c r="R18">
         <v>17</v>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="G19">
         <f>G17/C33</f>
-        <v>22.988972865740408</v>
+        <v>22.15054030497777</v>
       </c>
       <c r="R19" s="3">
         <v>18</v>
@@ -2604,11 +2604,11 @@
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="F20" s="15" t="s">
+      <c r="F20" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
       <c r="R20">
         <v>19</v>
       </c>
@@ -2623,7 +2623,7 @@
       </c>
       <c r="G21">
         <f>G18*2</f>
-        <v>74.293783743566024</v>
+        <v>71.584209561341794</v>
       </c>
       <c r="R21" s="3">
         <v>20</v>
@@ -2639,7 +2639,7 @@
       </c>
       <c r="G22">
         <f>G19*2</f>
-        <v>45.977945731480816</v>
+        <v>44.301080609955541</v>
       </c>
       <c r="R22">
         <v>21</v>
@@ -2653,11 +2653,11 @@
       <c r="B23" t="s">
         <v>58</v>
       </c>
-      <c r="F23" s="15" t="s">
+      <c r="F23" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
       <c r="R23">
         <v>22</v>
       </c>
@@ -2679,7 +2679,7 @@
       <c r="G24" s="10">
         <v>40</v>
       </c>
-      <c r="H24" s="18" t="s">
+      <c r="H24" s="16" t="s">
         <v>77</v>
       </c>
       <c r="I24">
@@ -2712,7 +2712,7 @@
       <c r="G25" s="10">
         <v>24</v>
       </c>
-      <c r="H25" s="18"/>
+      <c r="H25" s="16"/>
       <c r="I25">
         <v>15</v>
       </c>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="G26" s="6">
         <f>2*PI()*D4</f>
-        <v>512.07960253513625</v>
+        <v>502.6548245743669</v>
       </c>
       <c r="H26" s="6" t="s">
         <v>10</v>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="G27">
         <f>G26/G24</f>
-        <v>12.801990063378407</v>
+        <v>12.566370614359172</v>
       </c>
       <c r="H27" t="s">
         <v>10</v>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="G29">
         <f>G26/G25</f>
-        <v>21.336650105630678</v>
+        <v>20.943951023931955</v>
       </c>
       <c r="H29" t="s">
         <v>10</v>
@@ -3052,11 +3052,11 @@
       <c r="C37" t="s">
         <v>8</v>
       </c>
-      <c r="F37" s="19" t="s">
+      <c r="F37" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
+      <c r="G37" s="17"/>
+      <c r="H37" s="17"/>
       <c r="R37" s="3">
         <v>36</v>
       </c>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="G38">
         <f>B4</f>
-        <v>8.1500000000000003E-2</v>
+        <v>0.08</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="G43" s="11">
         <f>SQRT((3*(3+G41)*G39*G38^2)/(8*G42*G40))</f>
-        <v>1.093765748512995E-2</v>
+        <v>1.0736350905649032E-2</v>
       </c>
       <c r="H43" s="11" t="s">
         <v>11</v>
@@ -3163,7 +3163,7 @@
       </c>
       <c r="G44" s="1">
         <f>G43*1000</f>
-        <v>10.93765748512995</v>
+        <v>10.736350905649031</v>
       </c>
       <c r="H44" s="11" t="s">
         <v>10</v>
@@ -3175,11 +3175,11 @@
       <c r="H45" s="11"/>
     </row>
     <row r="46" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="F46" s="17" t="s">
+      <c r="F46" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="G46" s="17"/>
-      <c r="H46" s="17"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="13"/>
     </row>
     <row r="47" spans="1:19" x14ac:dyDescent="0.3">
       <c r="F47" s="11" t="s">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="G53" s="1">
         <f>G52-G44</f>
-        <v>24.987320851075619</v>
+        <v>25.188627430556537</v>
       </c>
       <c r="H53" s="11" t="s">
         <v>10</v>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="G54" s="1">
         <f>(PI()*(D14-G9-G44)^2*G53)/10^6</f>
-        <v>0.39521373560397088</v>
+        <v>0.40066152142546863</v>
       </c>
       <c r="H54" s="11" t="s">
         <v>3</v>
@@ -3277,7 +3277,7 @@
       </c>
       <c r="G55" s="1">
         <f>$D$10-2*G54</f>
-        <v>13.974673199932997</v>
+        <v>13.963777628290002</v>
       </c>
       <c r="H55" s="11" t="s">
         <v>3</v>
@@ -3300,7 +3300,7 @@
       </c>
       <c r="G57" s="1">
         <f>G55/(PI()*$B$4^2)</f>
-        <v>669.69425055159661</v>
+        <v>694.50132305574266</v>
       </c>
       <c r="H57" s="11" t="s">
         <v>10</v>
@@ -3312,25 +3312,25 @@
       </c>
       <c r="G58" s="1">
         <f>G57+2*(G56+35)</f>
-        <v>799.69425055159661</v>
+        <v>824.50132305574266</v>
       </c>
       <c r="H58" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="81" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G81" s="14" t="s">
+      <c r="G81" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="H81" s="14"/>
-      <c r="I81" s="14"/>
+      <c r="H81" s="15"/>
+      <c r="I81" s="15"/>
     </row>
     <row r="82" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G82" s="15" t="s">
+      <c r="G82" s="14" t="s">
         <v>103</v>
       </c>
-      <c r="H82" s="15"/>
-      <c r="I82" s="15"/>
+      <c r="H82" s="14"/>
+      <c r="I82" s="14"/>
     </row>
     <row r="83" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G83" t="s">
@@ -3353,7 +3353,7 @@
       <c r="I84" t="s">
         <v>8</v>
       </c>
-      <c r="J84" s="16" t="s">
+      <c r="J84" s="19" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       <c r="I85" t="s">
         <v>8</v>
       </c>
-      <c r="J85" s="16"/>
+      <c r="J85" s="19"/>
     </row>
     <row r="86" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G86" t="s">
@@ -3403,11 +3403,11 @@
       </c>
     </row>
     <row r="89" spans="7:11" x14ac:dyDescent="0.3">
-      <c r="G89" s="13" t="s">
+      <c r="G89" s="18" t="s">
         <v>111</v>
       </c>
-      <c r="H89" s="13"/>
-      <c r="I89" s="13"/>
+      <c r="H89" s="18"/>
+      <c r="I89" s="18"/>
     </row>
     <row r="90" spans="7:11" x14ac:dyDescent="0.3">
       <c r="G90" t="s">
@@ -3487,18 +3487,18 @@
       </c>
       <c r="H96" s="1">
         <f>H95/(PI()*$B$4^2)</f>
-        <v>607.53359258919409</v>
+        <v>630.5296883399335</v>
       </c>
       <c r="I96" s="11" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="98" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G98" s="13" t="s">
+      <c r="G98" s="18" t="s">
         <v>114</v>
       </c>
-      <c r="H98" s="13"/>
-      <c r="I98" s="13"/>
+      <c r="H98" s="18"/>
+      <c r="I98" s="18"/>
     </row>
     <row r="99" spans="7:9" x14ac:dyDescent="0.3">
       <c r="G99" t="s">
@@ -3574,7 +3574,7 @@
       </c>
       <c r="H105" s="1">
         <f>H104/(PI()*$B$4^2)</f>
-        <v>658.33430300321174</v>
+        <v>683.25328501923184</v>
       </c>
       <c r="I105" s="11" t="s">
         <v>10</v>
@@ -3582,6 +3582,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G98:I98"/>
+    <mergeCell ref="G81:I81"/>
+    <mergeCell ref="G82:I82"/>
+    <mergeCell ref="J84:J85"/>
+    <mergeCell ref="G89:I89"/>
     <mergeCell ref="F46:H46"/>
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="F23:H23"/>
@@ -3589,11 +3594,6 @@
     <mergeCell ref="F1:N1"/>
     <mergeCell ref="H24:H25"/>
     <mergeCell ref="F37:H37"/>
-    <mergeCell ref="G98:I98"/>
-    <mergeCell ref="G81:I81"/>
-    <mergeCell ref="G82:I82"/>
-    <mergeCell ref="J84:J85"/>
-    <mergeCell ref="G89:I89"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>